<commit_message>
Actualizacion automatica de datos - jue 04/06/2026 10:11:26,99
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA77BE94-1BB9-4B2B-B2D5-B490A572803A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId2"/>
+    <sheet name="Semana 2 - 8 al 14 Jun" sheetId="7" r:id="rId2"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="79">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -479,7 +480,327 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="64">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1130,25 +1451,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D799D698-03EA-4DEB-B560-23C342712620}">
-  <dimension ref="B2:L36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:L36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" style="2"/>
-    <col min="2" max="2" width="53.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5703125" style="2" bestFit="1"/>
-    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5703125" style="2" bestFit="1"/>
-    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5703125" style="2" bestFit="1"/>
-    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="4.5703125" style="2"/>
+    <col min="1" max="1" width="4.5546875" style="2"/>
+    <col min="2" max="2" width="53.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5546875" style="2" bestFit="1"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" style="2" bestFit="1"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.5546875" style="2" bestFit="1"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="4.5546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:12" ht="15" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" s="15" t="s">
         <v>68</v>
       </c>
@@ -1167,7 +1489,7 @@
       </c>
       <c r="L2" s="15"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -1194,7 +1516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1220,7 +1542,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -1246,7 +1568,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>67</v>
       </c>
@@ -1272,7 +1594,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -1298,7 +1620,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -1324,7 +1646,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -1350,7 +1672,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -1364,7 +1686,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="15" t="s">
         <v>69</v>
       </c>
@@ -1386,7 +1708,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -1412,7 +1734,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -1439,7 +1761,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -1466,7 +1788,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -1492,7 +1814,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -1508,7 +1830,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -1530,7 +1852,7 @@
       </c>
       <c r="L17" s="15"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="8" t="s">
         <v>61</v>
       </c>
@@ -1550,7 +1872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E19" s="15" t="s">
         <v>72</v>
       </c>
@@ -1568,7 +1890,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="15" t="s">
         <v>70</v>
       </c>
@@ -1592,7 +1914,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -1618,7 +1940,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="8" t="s">
         <v>27</v>
       </c>
@@ -1644,7 +1966,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="8" t="s">
         <v>29</v>
       </c>
@@ -1670,7 +1992,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="8" t="s">
         <v>31</v>
       </c>
@@ -1696,7 +2018,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="8" t="s">
         <v>32</v>
       </c>
@@ -1722,7 +2044,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>33</v>
       </c>
@@ -1742,7 +2064,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>20</v>
       </c>
@@ -1762,7 +2084,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>19</v>
       </c>
@@ -1782,7 +2104,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
         <v>35</v>
       </c>
@@ -1790,7 +2112,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
         <v>65</v>
       </c>
@@ -1806,7 +2128,7 @@
       </c>
       <c r="L30" s="15"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H31" s="13" t="s">
         <v>23</v>
       </c>
@@ -1820,7 +2142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="H32" s="5" t="s">
         <v>10</v>
       </c>
@@ -1834,7 +2156,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="8:12" x14ac:dyDescent="0.3">
       <c r="H33" s="5" t="s">
         <v>12</v>
       </c>
@@ -1848,7 +2170,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="8:12" x14ac:dyDescent="0.3">
       <c r="H34" s="5" t="s">
         <v>28</v>
       </c>
@@ -1862,7 +2184,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="8:12" x14ac:dyDescent="0.3">
       <c r="H35" s="5" t="s">
         <v>19</v>
       </c>
@@ -1876,7 +2198,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="8:12" x14ac:dyDescent="0.3">
       <c r="H36" s="5" t="s">
         <v>20</v>
       </c>
@@ -1893,114 +2215,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="31" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9 B29:B30">
-    <cfRule type="duplicateValues" dxfId="28" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="27" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B28">
-    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="21" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="20" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="19" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="18" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="16" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="15" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="13" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="12" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="11" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="7" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="6" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2008,15 +2330,892 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F9582F6-2340-4E7A-A61D-F0BEBF349FFA}">
+  <dimension ref="B2:L36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.5546875" style="2"/>
+    <col min="2" max="2" width="53.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5546875" style="2"/>
+    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" style="2"/>
+    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.5546875" style="2"/>
+    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="4.5546875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="H2" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="15"/>
+      <c r="K2" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="15"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="E11" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="15"/>
+      <c r="K17" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="L17" s="15"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E19" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" s="15"/>
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="E20" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" s="15"/>
+      <c r="K30" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="L30" s="15"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="8:12" x14ac:dyDescent="0.3">
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="8:12" x14ac:dyDescent="0.3">
+      <c r="H34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="8:12" x14ac:dyDescent="0.3">
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="8:12" x14ac:dyDescent="0.3">
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:B25">
+    <cfRule type="duplicateValues" dxfId="28" priority="48"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B26">
+    <cfRule type="duplicateValues" dxfId="27" priority="43"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30 B27 B9">
+    <cfRule type="duplicateValues" dxfId="26" priority="49"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="22" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24">
+    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="14" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="5" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -2024,7 +3223,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2032,7 +3231,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2040,7 +3239,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -2048,7 +3247,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -2056,7 +3255,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>19</v>
       </c>
@@ -2064,7 +3263,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
@@ -2072,7 +3271,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>44</v>
       </c>
@@ -2080,7 +3279,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
@@ -2088,7 +3287,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
@@ -2096,7 +3295,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
@@ -2104,7 +3303,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>62</v>
       </c>
@@ -2112,7 +3311,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>21</v>
       </c>
@@ -2120,7 +3319,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>49</v>
       </c>
@@ -2128,7 +3327,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>10</v>
       </c>
@@ -2136,7 +3335,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>27</v>
       </c>
@@ -2144,7 +3343,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>33</v>
       </c>
@@ -2152,7 +3351,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>31</v>
       </c>
@@ -2160,7 +3359,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
         <v>35</v>
       </c>
@@ -2168,7 +3367,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>29</v>
       </c>
@@ -2176,7 +3375,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>32</v>
       </c>
@@ -2184,7 +3383,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>28</v>
       </c>
@@ -2192,7 +3391,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>18</v>
       </c>
@@ -2200,7 +3399,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
         <v>11</v>
       </c>
@@ -2208,7 +3407,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>65</v>
       </c>
@@ -2223,8 +3422,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="850c2d3be926942608445a01d62c5196">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="62f8bdc36c683ccc6b5e07671bdc19f0" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
     <xsd:import namespace="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
     <xsd:element name="properties">
@@ -2297,7 +3496,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="fc5c7554-ce1a-493c-be4c-f5f61635795a" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -2316,7 +3515,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -2333,8 +3532,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2424,12 +3623,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2438,8 +3631,14 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0542880-A04A-4DC3-B5EC-DA1F7B46F86E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -2458,6 +3657,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -2472,12 +3679,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - lun 08/06/2026 11:24:39,71
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{565F7AE3-7BD4-421C-BBC1-1A8A9A0C43D1}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
@@ -480,7 +480,327 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="64">
+  <dxfs count="96">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2215,114 +2535,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="63" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="62" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="61" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9 B29:B30">
-    <cfRule type="duplicateValues" dxfId="60" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="59" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B28">
-    <cfRule type="duplicateValues" dxfId="58" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="57" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="56" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="55" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="54" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="53" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="52" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="51" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="50" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="48" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="47" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="46" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="45" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="44" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="43" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="39" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="38" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="37" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="36" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="35" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="34" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="33" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="32" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2335,17 +2655,17 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="4.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="2"/>
-    <col min="2" max="2" width="53.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.5546875" style="2"/>
-    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="4.5546875" style="2"/>
-    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="4.5546875" style="2"/>
-    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="4.5546875" style="2"/>
   </cols>
   <sheetData>
@@ -2400,25 +2720,25 @@
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>67</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>67</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.3">
@@ -2426,25 +2746,25 @@
         <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.3">
@@ -2452,25 +2772,25 @@
         <v>67</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
@@ -2478,25 +2798,25 @@
         <v>7</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>61</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>61</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -2504,25 +2824,25 @@
         <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
@@ -2530,25 +2850,25 @@
         <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
@@ -2556,13 +2876,13 @@
         <v>15</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>16</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
@@ -2578,13 +2898,13 @@
         <v>7</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
@@ -2604,13 +2924,13 @@
         <v>9</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="L12" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
@@ -2618,26 +2938,26 @@
         <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="L13" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
@@ -2645,26 +2965,26 @@
         <v>12</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="K14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L14" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
@@ -2672,25 +2992,25 @@
         <v>15</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>20</v>
       </c>
       <c r="L15" s="14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
@@ -2698,13 +3018,13 @@
         <v>21</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
@@ -2714,13 +3034,13 @@
         <v>22</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>74</v>
@@ -2736,7 +3056,7 @@
         <v>61</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>2</v>
@@ -2760,7 +3080,7 @@
         <v>10</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>10</v>
@@ -2784,13 +3104,13 @@
         <v>12</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K20" s="5" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
@@ -2804,19 +3124,19 @@
         <v>10</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.3">
@@ -2830,13 +3150,13 @@
         <v>12</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>6</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K22" s="5" t="s">
         <v>6</v>
@@ -2856,19 +3176,19 @@
         <v>28</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>15</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
@@ -2882,19 +3202,19 @@
         <v>19</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>7</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
@@ -2908,13 +3228,13 @@
         <v>20</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="K25" s="5" t="s">
         <v>9</v>
@@ -2934,13 +3254,13 @@
         <v>14</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>14</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
@@ -2954,13 +3274,13 @@
         <v>19</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>19</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
@@ -2974,13 +3294,13 @@
         <v>20</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K28" s="7" t="s">
         <v>20</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.3">
@@ -3026,13 +3346,13 @@
         <v>10</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="8:12" x14ac:dyDescent="0.3">
@@ -3040,13 +3360,13 @@
         <v>12</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>12</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="8:12" x14ac:dyDescent="0.3">
@@ -3054,13 +3374,13 @@
         <v>28</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K34" s="5" t="s">
         <v>28</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="8:12" x14ac:dyDescent="0.3">
@@ -3068,13 +3388,13 @@
         <v>19</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K35" s="5" t="s">
         <v>19</v>
       </c>
       <c r="L35" s="4" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="8:12" x14ac:dyDescent="0.3">
@@ -3082,59 +3402,59 @@
         <v>20</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K36" s="5" t="s">
         <v>20</v>
       </c>
       <c r="L36" s="4" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="31" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="28" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B26">
-    <cfRule type="duplicateValues" dxfId="27" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30 B27 B9">
-    <cfRule type="duplicateValues" dxfId="26" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
     <cfRule type="duplicateValues" dxfId="21" priority="16"/>
@@ -3158,7 +3478,7 @@
     <cfRule type="duplicateValues" dxfId="15" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
     <cfRule type="duplicateValues" dxfId="13" priority="11"/>
@@ -3185,7 +3505,7 @@
     <cfRule type="duplicateValues" dxfId="6" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
     <cfRule type="duplicateValues" dxfId="4" priority="8"/>
@@ -3422,6 +3742,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -3622,22 +3957,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3654,29 +3999,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - dom 14/06/2026 20:31:46,80
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{565F7AE3-7BD4-421C-BBC1-1A8A9A0C43D1}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5435C3C9-93D3-46F9-90FE-C66020B8CDFD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
     <sheet name="Semana 2 - 8 al 14 Jun" sheetId="7" r:id="rId2"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId3"/>
+    <sheet name="Semana 3 - 15 al 21" sheetId="8" r:id="rId3"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="80">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -303,6 +304,10 @@
   </si>
   <si>
     <t>Set 3 Domingo</t>
+  </si>
+  <si>
+    <t>Sebastian Hincapie / 
+Oriana</t>
   </si>
 </sst>
 </file>
@@ -345,11 +350,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -378,7 +385,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -427,11 +434,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -475,6 +506,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1771,26 +1820,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D799D698-03EA-4DEB-B560-23C342712620}">
-  <dimension ref="B1:L36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:L36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5546875" style="2"/>
-    <col min="2" max="2" width="53.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5546875" style="2" bestFit="1"/>
-    <col min="5" max="5" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5546875" style="2" bestFit="1"/>
-    <col min="8" max="8" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5546875" style="2" bestFit="1"/>
-    <col min="11" max="11" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="4.5546875" style="2"/>
+    <col min="1" max="1" width="4.5703125" style="2"/>
+    <col min="2" max="2" width="53.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" style="2" bestFit="1"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5703125" style="2" bestFit="1"/>
+    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.5703125" style="2" bestFit="1"/>
+    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="4.5703125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
         <v>68</v>
       </c>
@@ -1809,7 +1857,7 @@
       </c>
       <c r="L2" s="15"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -1836,7 +1884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1862,7 +1910,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -1888,7 +1936,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>67</v>
       </c>
@@ -1914,7 +1962,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -1940,7 +1988,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -1966,7 +2014,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -1992,7 +2040,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -2006,7 +2054,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="15" t="s">
         <v>69</v>
       </c>
@@ -2028,7 +2076,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -2054,7 +2102,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -2081,7 +2129,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -2108,7 +2156,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -2134,7 +2182,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -2150,7 +2198,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -2172,7 +2220,7 @@
       </c>
       <c r="L17" s="15"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>61</v>
       </c>
@@ -2192,7 +2240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E19" s="15" t="s">
         <v>72</v>
       </c>
@@ -2210,7 +2258,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>70</v>
       </c>
@@ -2234,7 +2282,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -2260,7 +2308,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
         <v>27</v>
       </c>
@@ -2286,7 +2334,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
         <v>29</v>
       </c>
@@ -2312,7 +2360,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>31</v>
       </c>
@@ -2338,7 +2386,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>32</v>
       </c>
@@ -2364,7 +2412,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>33</v>
       </c>
@@ -2384,7 +2432,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
         <v>20</v>
       </c>
@@ -2404,7 +2452,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
         <v>19</v>
       </c>
@@ -2424,7 +2472,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
         <v>35</v>
       </c>
@@ -2432,7 +2480,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="5" t="s">
         <v>65</v>
       </c>
@@ -2448,7 +2496,7 @@
       </c>
       <c r="L30" s="15"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
         <v>23</v>
       </c>
@@ -2462,7 +2510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H32" s="5" t="s">
         <v>10</v>
       </c>
@@ -2476,7 +2524,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H33" s="5" t="s">
         <v>12</v>
       </c>
@@ -2490,7 +2538,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H34" s="5" t="s">
         <v>28</v>
       </c>
@@ -2504,7 +2552,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H35" s="5" t="s">
         <v>19</v>
       </c>
@@ -2518,7 +2566,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H36" s="5" t="s">
         <v>20</v>
       </c>
@@ -2535,18 +2583,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="40"/>
@@ -2652,24 +2700,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F9582F6-2340-4E7A-A61D-F0BEBF349FFA}">
   <dimension ref="B2:L36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="4.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5546875" style="2"/>
-    <col min="2" max="2" width="52.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5546875" style="2"/>
-    <col min="5" max="5" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5546875" style="2"/>
-    <col min="8" max="8" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.5703125" style="2"/>
+    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" style="2"/>
+    <col min="5" max="5" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5703125" style="2"/>
+    <col min="8" max="8" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5546875" style="2"/>
-    <col min="11" max="11" width="46.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="4.5546875" style="2"/>
+    <col min="10" max="10" width="4.5703125" style="2"/>
+    <col min="11" max="11" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="4.5703125" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
         <v>68</v>
       </c>
@@ -2688,7 +2736,7 @@
       </c>
       <c r="L2" s="15"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
@@ -2715,7 +2763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
@@ -2741,7 +2789,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
@@ -2767,7 +2815,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>67</v>
       </c>
@@ -2793,7 +2841,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
@@ -2819,7 +2867,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
@@ -2845,7 +2893,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
@@ -2871,7 +2919,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -2885,7 +2933,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="15" t="s">
         <v>69</v>
       </c>
@@ -2907,7 +2955,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="13" t="s">
         <v>0</v>
       </c>
@@ -2933,7 +2981,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
@@ -2960,7 +3008,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
@@ -2987,7 +3035,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -3013,7 +3061,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -3029,7 +3077,7 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
@@ -3051,7 +3099,7 @@
       </c>
       <c r="L17" s="15"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
         <v>61</v>
       </c>
@@ -3071,7 +3119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E19" s="15" t="s">
         <v>72</v>
       </c>
@@ -3089,7 +3137,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>70</v>
       </c>
@@ -3113,7 +3161,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="13" t="s">
         <v>0</v>
       </c>
@@ -3139,7 +3187,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="8" t="s">
         <v>29</v>
       </c>
@@ -3165,7 +3213,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
         <v>31</v>
       </c>
@@ -3191,7 +3239,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>27</v>
       </c>
@@ -3217,7 +3265,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>32</v>
       </c>
@@ -3243,7 +3291,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>20</v>
       </c>
@@ -3263,7 +3311,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
         <v>35</v>
       </c>
@@ -3283,7 +3331,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
         <v>33</v>
       </c>
@@ -3303,7 +3351,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
         <v>19</v>
       </c>
@@ -3311,7 +3359,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="5" t="s">
         <v>65</v>
       </c>
@@ -3327,7 +3375,7 @@
       </c>
       <c r="L30" s="15"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
         <v>23</v>
       </c>
@@ -3341,7 +3389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H32" s="5" t="s">
         <v>10</v>
       </c>
@@ -3355,7 +3403,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H33" s="5" t="s">
         <v>12</v>
       </c>
@@ -3369,7 +3417,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H34" s="5" t="s">
         <v>28</v>
       </c>
@@ -3383,7 +3431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H35" s="5" t="s">
         <v>19</v>
       </c>
@@ -3397,7 +3445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="8:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H36" s="5" t="s">
         <v>20</v>
       </c>
@@ -3409,14 +3457,897 @@
       </c>
       <c r="L36" s="4" t="s">
         <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="63" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:B25">
+    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B26">
+    <cfRule type="duplicateValues" dxfId="59" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30 B27 B9">
+    <cfRule type="duplicateValues" dxfId="58" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="55" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24">
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="35" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="34" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="32" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A9D3091-ADE9-4FBE-947A-243F060C2AE5}">
+  <dimension ref="B2:L36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="2"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="2"/>
+    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="2"/>
+    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="H2" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="15"/>
+      <c r="K2" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="15"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="E11" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="15"/>
+      <c r="K17" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="L17" s="15"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="17" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="E20" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="15"/>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K28" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" s="15"/>
+      <c r="K30" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="L30" s="15"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="H34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
     <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
@@ -3462,10 +4393,10 @@
   <conditionalFormatting sqref="E17">
     <cfRule type="duplicateValues" dxfId="20" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E24">
+  <conditionalFormatting sqref="E25">
     <cfRule type="duplicateValues" dxfId="19" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E25">
+  <conditionalFormatting sqref="E26">
     <cfRule type="duplicateValues" dxfId="18" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
@@ -3526,16 +4457,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="95.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -3543,7 +4474,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
@@ -3551,7 +4482,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3559,7 +4490,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -3567,7 +4498,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -3575,7 +4506,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>19</v>
       </c>
@@ -3583,7 +4514,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
@@ -3591,7 +4522,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>44</v>
       </c>
@@ -3599,7 +4530,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
@@ -3607,7 +4538,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
@@ -3615,7 +4546,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
@@ -3623,7 +4554,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>62</v>
       </c>
@@ -3631,7 +4562,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>21</v>
       </c>
@@ -3639,7 +4570,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>49</v>
       </c>
@@ -3647,7 +4578,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>10</v>
       </c>
@@ -3655,7 +4586,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>27</v>
       </c>
@@ -3663,7 +4594,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>33</v>
       </c>
@@ -3671,7 +4602,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>31</v>
       </c>
@@ -3679,7 +4610,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>35</v>
       </c>
@@ -3687,7 +4618,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="144" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>29</v>
       </c>
@@ -3695,7 +4626,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>32</v>
       </c>
@@ -3703,7 +4634,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>28</v>
       </c>
@@ -3711,7 +4642,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>18</v>
       </c>
@@ -3719,7 +4650,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>11</v>
       </c>
@@ -3727,7 +4658,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>65</v>
       </c>
@@ -3742,21 +4673,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -3957,32 +4873,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3999,4 +4905,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Cronograma Junio.xlsx with new changes from user
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5435C3C9-93D3-46F9-90FE-C66020B8CDFD}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41A69BDD-4038-4B08-930D-FD6C9E010B74}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="79">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -304,10 +304,6 @@
   </si>
   <si>
     <t>Set 3 Domingo</t>
-  </si>
-  <si>
-    <t>Sebastian Hincapie / 
-Oriana</t>
   </si>
 </sst>
 </file>
@@ -504,9 +500,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -524,6 +517,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1839,23 +1835,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="21"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="H2" s="15" t="s">
+      <c r="F2" s="21"/>
+      <c r="H2" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="15"/>
-      <c r="K2" s="15" t="s">
+      <c r="I2" s="21"/>
+      <c r="K2" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="15"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -2055,14 +2051,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="E11" s="15" t="s">
+      <c r="C11" s="21"/>
+      <c r="E11" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="15"/>
+      <c r="F11" s="21"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -2211,14 +2207,14 @@
       <c r="F17" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="15"/>
-      <c r="K17" s="15" t="s">
+      <c r="I17" s="21"/>
+      <c r="K17" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="15"/>
+      <c r="L17" s="21"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -2241,10 +2237,10 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="F19" s="15"/>
+      <c r="F19" s="21"/>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2259,10 +2255,10 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="15"/>
+      <c r="C20" s="21"/>
       <c r="E20" s="13" t="s">
         <v>23</v>
       </c>
@@ -2487,14 +2483,14 @@
       <c r="C30" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="H30" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="15"/>
-      <c r="K30" s="15" t="s">
+      <c r="I30" s="21"/>
+      <c r="K30" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="15"/>
+      <c r="L30" s="21"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -2583,18 +2579,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="40"/>
@@ -2718,23 +2714,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="21"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="H2" s="15" t="s">
+      <c r="F2" s="21"/>
+      <c r="H2" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="15"/>
-      <c r="K2" s="15" t="s">
+      <c r="I2" s="21"/>
+      <c r="K2" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="15"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -2934,14 +2930,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="E11" s="15" t="s">
+      <c r="C11" s="21"/>
+      <c r="E11" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="15"/>
+      <c r="F11" s="21"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -3090,14 +3086,14 @@
       <c r="F17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="15"/>
-      <c r="K17" s="15" t="s">
+      <c r="I17" s="21"/>
+      <c r="K17" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="15"/>
+      <c r="L17" s="21"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -3120,10 +3116,10 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="F19" s="15"/>
+      <c r="F19" s="21"/>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -3138,10 +3134,10 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="15"/>
+      <c r="C20" s="21"/>
       <c r="E20" s="13" t="s">
         <v>23</v>
       </c>
@@ -3366,14 +3362,14 @@
       <c r="C30" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="H30" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="15"/>
-      <c r="K30" s="15" t="s">
+      <c r="I30" s="21"/>
+      <c r="K30" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="15"/>
+      <c r="L30" s="21"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -3461,18 +3457,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="63" priority="29"/>
@@ -3595,23 +3591,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="21"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="H2" s="15" t="s">
+      <c r="F2" s="21"/>
+      <c r="H2" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="15"/>
-      <c r="K2" s="15" t="s">
+      <c r="I2" s="21"/>
+      <c r="K2" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="15"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -3811,14 +3807,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="E11" s="15" t="s">
+      <c r="C11" s="21"/>
+      <c r="E11" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="15"/>
+      <c r="F11" s="21"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -3912,7 +3908,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>15</v>
       </c>
@@ -3922,8 +3918,8 @@
       <c r="E15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="16" t="s">
-        <v>79</v>
+      <c r="F15" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>20</v>
@@ -3946,10 +3942,10 @@
         <v>24</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>30</v>
+        <v>18</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
@@ -3962,19 +3958,19 @@
         <v>24</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="15"/>
-      <c r="K17" s="15" t="s">
+      <c r="I17" s="21"/>
+      <c r="K17" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="15"/>
+      <c r="L17" s="21"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -3984,10 +3980,10 @@
         <v>24</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>2</v>
@@ -3998,18 +3994,24 @@
       <c r="K18" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="L18" s="17" t="s">
+      <c r="L18" s="16" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K19" s="18" t="s">
+      <c r="K19" s="17" t="s">
         <v>10</v>
       </c>
       <c r="L19" s="4" t="s">
@@ -4017,21 +4019,17 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="E20" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="F20" s="15"/>
+      <c r="C20" s="21"/>
       <c r="H20" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K20" s="18" t="s">
+      <c r="K20" s="17" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="4" t="s">
@@ -4045,19 +4043,17 @@
       <c r="C21" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>1</v>
-      </c>
+      <c r="E21" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" s="21"/>
       <c r="H21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="19" t="s">
+      <c r="K21" s="18" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="4" t="s">
@@ -4071,11 +4067,11 @@
       <c r="C22" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>4</v>
+      <c r="E22" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>1</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>6</v>
@@ -4083,7 +4079,7 @@
       <c r="I22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K22" s="18" t="s">
+      <c r="K22" s="17" t="s">
         <v>6</v>
       </c>
       <c r="L22" s="4" t="s">
@@ -4098,7 +4094,7 @@
         <v>30</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>4</v>
@@ -4109,7 +4105,7 @@
       <c r="I23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="K23" s="17" t="s">
         <v>15</v>
       </c>
       <c r="L23" s="4" t="s">
@@ -4124,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>4</v>
@@ -4135,7 +4131,7 @@
       <c r="I24" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K24" s="18" t="s">
+      <c r="K24" s="17" t="s">
         <v>7</v>
       </c>
       <c r="L24" s="4" t="s">
@@ -4150,7 +4146,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>4</v>
@@ -4161,7 +4157,7 @@
       <c r="I25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="K25" s="17" t="s">
         <v>9</v>
       </c>
       <c r="L25" s="4" t="s">
@@ -4176,7 +4172,7 @@
         <v>25</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>4</v>
@@ -4187,7 +4183,7 @@
       <c r="I26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="K26" s="17" t="s">
         <v>14</v>
       </c>
       <c r="L26" s="4" t="s">
@@ -4201,13 +4197,19 @@
       <c r="C27" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="E27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="H27" s="6" t="s">
         <v>19</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K27" s="20" t="s">
+      <c r="K27" s="19" t="s">
         <v>19</v>
       </c>
       <c r="L27" s="4" t="s">
@@ -4227,7 +4229,7 @@
       <c r="I28" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K28" s="21" t="s">
+      <c r="K28" s="20" t="s">
         <v>20</v>
       </c>
       <c r="L28" s="4" t="s">
@@ -4249,14 +4251,14 @@
       <c r="C30" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="H30" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="15"/>
-      <c r="K30" s="15" t="s">
+      <c r="I30" s="21"/>
+      <c r="K30" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="15"/>
+      <c r="L30" s="21"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -4344,18 +4346,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="29"/>
@@ -4387,16 +4389,16 @@
   <conditionalFormatting sqref="E9">
     <cfRule type="duplicateValues" dxfId="22" priority="26"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E16">
+  <conditionalFormatting sqref="E17">
     <cfRule type="duplicateValues" dxfId="21" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E17">
+  <conditionalFormatting sqref="E18">
     <cfRule type="duplicateValues" dxfId="20" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E25">
+  <conditionalFormatting sqref="E26">
     <cfRule type="duplicateValues" dxfId="19" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E26">
+  <conditionalFormatting sqref="E27">
     <cfRule type="duplicateValues" dxfId="18" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
@@ -4673,6 +4675,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -4873,22 +4890,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4905,29 +4932,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Cronograma Junio.xlsx with latest changes from user
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41A69BDD-4038-4B08-930D-FD6C9E010B74}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B60C7082-D2A8-49B6-B459-49BC286C4A2B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="79">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -458,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -499,9 +499,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1835,23 +1832,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="21"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="H2" s="21" t="s">
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="21"/>
-      <c r="K2" s="21" t="s">
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="20"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -2051,14 +2048,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="E11" s="21" t="s">
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="21"/>
+      <c r="F11" s="20"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -2207,14 +2204,14 @@
       <c r="F17" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="21" t="s">
+      <c r="H17" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="21"/>
-      <c r="K17" s="21" t="s">
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="21"/>
+      <c r="L17" s="20"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -2237,10 +2234,10 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="21" t="s">
+      <c r="E19" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F19" s="21"/>
+      <c r="F19" s="20"/>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -2255,10 +2252,10 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="20"/>
       <c r="E20" s="13" t="s">
         <v>23</v>
       </c>
@@ -2483,14 +2480,14 @@
       <c r="C30" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H30" s="21" t="s">
+      <c r="H30" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="21"/>
-      <c r="K30" s="21" t="s">
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="21"/>
+      <c r="L30" s="20"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -2579,18 +2576,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="40"/>
@@ -2714,23 +2711,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="21"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="H2" s="21" t="s">
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="21"/>
-      <c r="K2" s="21" t="s">
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="20"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -2930,14 +2927,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="E11" s="21" t="s">
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="21"/>
+      <c r="F11" s="20"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -3086,14 +3083,14 @@
       <c r="F17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="21" t="s">
+      <c r="H17" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="21"/>
-      <c r="K17" s="21" t="s">
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="21"/>
+      <c r="L17" s="20"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -3116,10 +3113,10 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="21" t="s">
+      <c r="E19" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F19" s="21"/>
+      <c r="F19" s="20"/>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -3134,10 +3131,10 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="20"/>
       <c r="E20" s="13" t="s">
         <v>23</v>
       </c>
@@ -3362,14 +3359,14 @@
       <c r="C30" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H30" s="21" t="s">
+      <c r="H30" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="21"/>
-      <c r="K30" s="21" t="s">
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="21"/>
+      <c r="L30" s="20"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -3457,18 +3454,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="63" priority="29"/>
@@ -3591,23 +3588,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="21"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="H2" s="21" t="s">
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="21"/>
-      <c r="K2" s="21" t="s">
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="20"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
@@ -3807,14 +3804,14 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="E11" s="21" t="s">
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="21"/>
+      <c r="F11" s="20"/>
       <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
@@ -3866,7 +3863,7 @@
         <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>14</v>
@@ -3893,7 +3890,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>19</v>
@@ -3918,8 +3915,8 @@
       <c r="E15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>17</v>
+      <c r="F15" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>20</v>
@@ -3944,8 +3941,8 @@
       <c r="E16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>34</v>
+      <c r="F16" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
@@ -3961,16 +3958,16 @@
         <v>19</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H17" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="H17" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="I17" s="21"/>
-      <c r="K17" s="21" t="s">
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="L17" s="21"/>
+      <c r="L17" s="20"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
@@ -3983,7 +3980,7 @@
         <v>20</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>2</v>
@@ -3994,7 +3991,7 @@
       <c r="K18" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="L18" s="16" t="s">
+      <c r="L18" s="15" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4011,7 +4008,7 @@
       <c r="I19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="K19" s="16" t="s">
         <v>10</v>
       </c>
       <c r="L19" s="4" t="s">
@@ -4019,17 +4016,17 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="20"/>
       <c r="H20" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="K20" s="16" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="4" t="s">
@@ -4043,17 +4040,17 @@
       <c r="C21" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="21" t="s">
+      <c r="E21" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F21" s="21"/>
+      <c r="F21" s="20"/>
       <c r="H21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="K21" s="17" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="4" t="s">
@@ -4079,7 +4076,7 @@
       <c r="I22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="K22" s="16" t="s">
         <v>6</v>
       </c>
       <c r="L22" s="4" t="s">
@@ -4105,7 +4102,7 @@
       <c r="I23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K23" s="17" t="s">
+      <c r="K23" s="16" t="s">
         <v>15</v>
       </c>
       <c r="L23" s="4" t="s">
@@ -4131,7 +4128,7 @@
       <c r="I24" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K24" s="17" t="s">
+      <c r="K24" s="16" t="s">
         <v>7</v>
       </c>
       <c r="L24" s="4" t="s">
@@ -4157,7 +4154,7 @@
       <c r="I25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K25" s="17" t="s">
+      <c r="K25" s="16" t="s">
         <v>9</v>
       </c>
       <c r="L25" s="4" t="s">
@@ -4183,7 +4180,7 @@
       <c r="I26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K26" s="17" t="s">
+      <c r="K26" s="16" t="s">
         <v>14</v>
       </c>
       <c r="L26" s="4" t="s">
@@ -4209,7 +4206,7 @@
       <c r="I27" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K27" s="19" t="s">
+      <c r="K27" s="18" t="s">
         <v>19</v>
       </c>
       <c r="L27" s="4" t="s">
@@ -4218,10 +4215,10 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>20</v>
@@ -4229,7 +4226,7 @@
       <c r="I28" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K28" s="20" t="s">
+      <c r="K28" s="19" t="s">
         <v>20</v>
       </c>
       <c r="L28" s="4" t="s">
@@ -4238,27 +4235,21 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H30" s="21" t="s">
+      <c r="H30" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="21"/>
-      <c r="K30" s="21" t="s">
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="L30" s="21"/>
+      <c r="L30" s="20"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H31" s="13" t="s">
@@ -4346,18 +4337,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="29"/>
@@ -4371,10 +4362,10 @@
   <conditionalFormatting sqref="B22:B25">
     <cfRule type="duplicateValues" dxfId="28" priority="31"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B29 B26">
+  <conditionalFormatting sqref="B28 B26">
     <cfRule type="duplicateValues" dxfId="27" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30 B27 B9">
+  <conditionalFormatting sqref="B29 B27 B9">
     <cfRule type="duplicateValues" dxfId="26" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
@@ -4675,21 +4666,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -4890,32 +4866,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4932,4 +4898,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix uid error and update chart data
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B60C7082-D2A8-49B6-B459-49BC286C4A2B}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB5B6EC4-BBB5-46CA-A7F5-A5F775256843}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
@@ -2576,18 +2576,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="40"/>
@@ -2699,8 +2699,8 @@
     <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.5703125" style="2"/>
-    <col min="5" max="5" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="4.5703125" style="2"/>
     <col min="8" max="8" width="46.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" style="2" bestFit="1" customWidth="1"/>
@@ -3454,18 +3454,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="63" priority="29"/>
@@ -4337,18 +4337,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="29"/>
@@ -4666,6 +4666,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -4866,22 +4881,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4898,29 +4923,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 19/06/2026 18:14:48,12
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB5B6EC4-BBB5-46CA-A7F5-A5F775256843}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AC3D8D1-F3A3-4181-9AEE-865E365D393D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
     <sheet name="Semana 2 - 8 al 14 Jun" sheetId="7" r:id="rId2"/>
     <sheet name="Semana 3 - 15 al 21" sheetId="8" r:id="rId3"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId4"/>
+    <sheet name="Semana 4 - 22 al 28 Jun" sheetId="9" r:id="rId4"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="80">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -304,6 +305,9 @@
   </si>
   <si>
     <t>Set 3 Domingo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josue </t>
   </si>
 </sst>
 </file>
@@ -522,7 +526,327 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="96">
+  <dxfs count="128">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2576,114 +2900,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="95" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="94" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="93" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9 B29:B30">
-    <cfRule type="duplicateValues" dxfId="92" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="91" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B28">
-    <cfRule type="duplicateValues" dxfId="90" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="89" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="88" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="87" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="86" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="85" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="84" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="83" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="82" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="80" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="79" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="78" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="77" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="76" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="75" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="74" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="73" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="72" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="71" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="70" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="69" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="68" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="67" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="66" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="65" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="64" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3454,114 +3778,114 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="63" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B26">
-    <cfRule type="duplicateValues" dxfId="59" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30 B27 B9">
-    <cfRule type="duplicateValues" dxfId="58" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="55" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="35" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="34" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="32" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4337,120 +4661,1043 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="29" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B26">
-    <cfRule type="duplicateValues" dxfId="27" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B27 B9">
-    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F909C4A7-11F5-4C4B-ADFC-ADF85872A167}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="2"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="2"/>
+    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="2"/>
+    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L17" s="20"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="E20" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="20"/>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="L30" s="20"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="H34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="29" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:B25">
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B26">
+    <cfRule type="duplicateValues" dxfId="27" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30 B27 B9">
+    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25">
+    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="14" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4666,21 +5913,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -4881,32 +6113,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4923,4 +6145,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - mar 23/06/2026  9:04:05,71
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AC3D8D1-F3A3-4181-9AEE-865E365D393D}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA6074F0-DD8A-429E-9B7E-47D262E55BE7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="81">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t xml:space="preserve">Josue </t>
+  </si>
+  <si>
+    <t>Luis</t>
   </si>
 </sst>
 </file>
@@ -2900,18 +2903,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="127" priority="40"/>
@@ -3778,18 +3781,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="29"/>
@@ -4661,18 +4664,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="63" priority="29"/>
@@ -4776,7 +4779,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F909C4A7-11F5-4C4B-ADFC-ADF85872A167}">
-  <dimension ref="B2:L41"/>
+  <dimension ref="B2:L42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
@@ -4897,7 +4900,7 @@
         <v>67</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>7</v>
@@ -4975,7 +4978,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>14</v>
@@ -4997,6 +5000,12 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
@@ -5011,10 +5020,6 @@
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C11" s="20"/>
       <c r="E11" s="20" t="s">
         <v>71</v>
       </c>
@@ -5033,12 +5038,10 @@
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>1</v>
-      </c>
+      <c r="B12" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="20"/>
       <c r="E12" s="13" t="s">
         <v>2</v>
       </c>
@@ -5059,11 +5062,11 @@
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>5</v>
+      <c r="B13" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>1</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="5" t="s">
@@ -5087,7 +5090,7 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>5</v>
@@ -5114,7 +5117,7 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>5</v>
@@ -5140,7 +5143,7 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>5</v>
@@ -5154,9 +5157,9 @@
       <c r="I16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="B17" s="12" t="s">
-        <v>22</v>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>5</v>
@@ -5176,9 +5179,9 @@
       </c>
       <c r="L17" s="20"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="8" t="s">
-        <v>61</v>
+    <row r="18" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B18" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>5</v>
@@ -5203,6 +5206,12 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>10</v>
       </c>
@@ -5217,10 +5226,6 @@
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="20"/>
       <c r="E20" s="20" t="s">
         <v>72</v>
       </c>
@@ -5239,12 +5244,10 @@
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>1</v>
-      </c>
+      <c r="B21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="20"/>
       <c r="E21" s="13" t="s">
         <v>23</v>
       </c>
@@ -5265,11 +5268,11 @@
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>17</v>
+      <c r="B22" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>10</v>
@@ -5292,7 +5295,7 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>17</v>
@@ -5318,10 +5321,10 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>28</v>
@@ -5344,7 +5347,7 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>60</v>
@@ -5369,8 +5372,8 @@
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="5" t="s">
-        <v>20</v>
+      <c r="B26" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>60</v>
@@ -5396,7 +5399,7 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>60</v>
@@ -5416,10 +5419,10 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>20</v>
@@ -5436,18 +5439,18 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="5" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="H30" s="20" t="s">
         <v>75</v>
@@ -5459,6 +5462,12 @@
       <c r="L30" s="20"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="H31" s="13" t="s">
         <v>23</v>
       </c>
@@ -5473,8 +5482,6 @@
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B32"/>
-      <c r="C32"/>
       <c r="D32"/>
       <c r="H32" s="5" t="s">
         <v>10</v>
@@ -5582,20 +5589,24 @@
       <c r="C41"/>
       <c r="D41"/>
     </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B42"/>
+      <c r="C42"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="29"/>
@@ -5606,13 +5617,13 @@
   <conditionalFormatting sqref="B8">
     <cfRule type="duplicateValues" dxfId="29" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B22:B25">
+  <conditionalFormatting sqref="B23:B26">
     <cfRule type="duplicateValues" dxfId="28" priority="31"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B29 B26">
+  <conditionalFormatting sqref="B30 B27">
     <cfRule type="duplicateValues" dxfId="27" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30 B27 B9">
+  <conditionalFormatting sqref="B31 B28 B9">
     <cfRule type="duplicateValues" dxfId="26" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
@@ -5913,6 +5924,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -6113,22 +6139,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6145,29 +6181,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 26/06/2026 15:13:42,16
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA6074F0-DD8A-429E-9B7E-47D262E55BE7}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D1BEF34-2ABD-4318-9D87-5BC5000EB959}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Semana 1 - 1 al 7 Jun" sheetId="6" r:id="rId1"/>
     <sheet name="Semana 2 - 8 al 14 Jun" sheetId="7" r:id="rId2"/>
     <sheet name="Semana 3 - 15 al 21" sheetId="8" r:id="rId3"/>
     <sheet name="Semana 4 - 22 al 28 Jun" sheetId="9" r:id="rId4"/>
-    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId5"/>
+    <sheet name="Semana 5 - 29 Jun al 5 de Jul" sheetId="10" r:id="rId5"/>
+    <sheet name="Detalle Cronograma" sheetId="2" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="82">
   <si>
     <t>Cronograma Mañana</t>
   </si>
@@ -311,6 +312,9 @@
   </si>
   <si>
     <t>Luis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan Jose </t>
   </si>
 </sst>
 </file>
@@ -529,7 +533,327 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="128">
+  <dxfs count="160">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2903,114 +3227,114 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="127" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="126" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="125" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9 B29:B30">
-    <cfRule type="duplicateValues" dxfId="124" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="123" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:B28">
-    <cfRule type="duplicateValues" dxfId="122" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="121" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="120" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="119" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="151" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="118" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="117" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="116" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="115" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="114" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="113" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="112" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="111" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="110" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="109" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="108" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="107" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="106" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="105" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="104" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="103" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="102" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="101" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="100" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="99" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="98" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="97" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="96" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3781,114 +4105,114 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="95" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="94" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="93" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="92" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B26">
-    <cfRule type="duplicateValues" dxfId="91" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30 B27 B9">
-    <cfRule type="duplicateValues" dxfId="90" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="89" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="88" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="87" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="86" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16">
-    <cfRule type="duplicateValues" dxfId="85" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="84" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24">
-    <cfRule type="duplicateValues" dxfId="83" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="82" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="80" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="79" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="78" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="77" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="76" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="75" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="73" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="72" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="71" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="70" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="69" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="68" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="67" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="66" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="65" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="64" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4664,114 +4988,114 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="63" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B25">
-    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28 B26">
-    <cfRule type="duplicateValues" dxfId="59" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29 B27 B9">
-    <cfRule type="duplicateValues" dxfId="58" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="55" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27">
-    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="35" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="34" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="32" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5595,120 +5919,1043 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="29" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B26">
-    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30 B27">
-    <cfRule type="duplicateValues" dxfId="27" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31 B28 B9">
-    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6">
-    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9">
-    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17">
-    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18">
-    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25">
-    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26">
-    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
-    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="duplicateValues" dxfId="14" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H24">
-    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H25">
-    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35">
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H36">
-    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K24">
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K35">
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C7291A-7212-4757-A43C-50195386FDB5}">
+  <dimension ref="B2:L41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="2"/>
+    <col min="5" max="5" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="2"/>
+    <col min="8" max="8" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="2"/>
+    <col min="11" max="11" width="52.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="15" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="20"/>
+      <c r="H2" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="20"/>
+      <c r="K2" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="E11" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="20"/>
+      <c r="K17" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L17" s="20"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="H20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" s="20"/>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K28" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H30" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" s="20"/>
+      <c r="K30" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="L30" s="20"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="H32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="H33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="H34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="H35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="duplicateValues" dxfId="29" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:B25">
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28 B26">
+    <cfRule type="duplicateValues" dxfId="27" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29 B27 B9">
+    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27">
+    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="duplicateValues" dxfId="14" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="duplicateValues" dxfId="7" priority="18"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
+    <cfRule type="duplicateValues" dxfId="5" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25">
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K26">
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K36">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EE4785-03B3-42C8-BF36-D812A392D9B8}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="95.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5924,21 +7171,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -6139,32 +7371,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6181,4 +7403,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C882070A-3085-4CEC-A419-8DBCE0B99BE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="fc5c7554-ce1a-493c-be4c-f5f61635795a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 10/07/2026 14:46:45,64
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Junio.xlsx
+++ b/Cronograma de Tareas/Cronograma Junio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Cronograma de Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D1BEF34-2ABD-4318-9D87-5BC5000EB959}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{06FAC02E-6217-4A13-88B2-5364F8FE09FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CB7E2E9-88A0-4EB1-AD67-9FAF11CCE993}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{F65F8D10-F9E7-465F-B378-86A66F7EDF21}"/>
   </bookViews>
@@ -3227,18 +3227,18 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="luPs9DkHAzoolt26JtBUVTn7qgShzp51GTfA8y1cPBsZ9eHrMBxBJVPqoRpJ9W0yLl67bfaElIfQgtUGsZrhOA==" saltValue="7CKQnFDspZDX2lb1Mzl6Ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="159" priority="40"/>
@@ -4105,18 +4105,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="127" priority="29"/>
@@ -4988,18 +4988,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="95" priority="29"/>
@@ -5919,18 +5919,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="63" priority="29"/>
@@ -6477,7 +6477,7 @@
         <v>10</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
@@ -6519,7 +6519,7 @@
         <v>3</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
@@ -6571,7 +6571,7 @@
         <v>15</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
@@ -6623,7 +6623,7 @@
         <v>9</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
@@ -6675,7 +6675,7 @@
         <v>19</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
@@ -6842,18 +6842,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="29"/>
@@ -7171,6 +7171,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DF699C9B971E44AADE72149239363A2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd28a159404b63a0ef222e938afe2db3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ef2aad6-6696-4ad1-83da-256baa9d6106" xmlns:ns3="fc5c7554-ce1a-493c-be4c-f5f61635795a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b25b72c149c8f1dd75cad995c7ef7c98" ns2:_="" ns3:_="">
     <xsd:import namespace="3ef2aad6-6696-4ad1-83da-256baa9d6106"/>
@@ -7371,15 +7380,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -7387,6 +7387,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00384C4C-6C78-4D12-9861-ADDC632264D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7401,14 +7409,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6ADFC66-A3DD-491F-9CEF-E18565F39C8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>